<commit_message>
Correções do script do banco de dados
Agora realizando a avaliação de acordo com o pretendido.
</commit_message>
<xml_diff>
--- a/avaliacao.xlsx
+++ b/avaliacao.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Avaliação" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -46,7 +46,7 @@
     <t>Artigo completo publicado em periódico especializado, com Qualis</t>
   </si>
   <si>
-    <t>Artigo completo publicado em periódico especializado, sem Qualis</t>
+    <t xml:space="preserve">Artigo completo publicado em periódico especializado, sem Qualis </t>
   </si>
   <si>
     <t>Trabalhos completos publicados em Anais, em evento local, regional, nacional ou internacional.</t>
@@ -85,8 +85,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,13 +149,18 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Escritório">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -193,7 +198,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Escritório">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -227,6 +232,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -261,9 +267,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Escritório">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -436,11 +443,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="30.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -460,7 +470,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -480,7 +490,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -500,7 +510,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -517,10 +527,10 @@
         <v>2</v>
       </c>
       <c r="F4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -534,33 +544,33 @@
         <v>3999996</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>3999996</v>
+        <v>1999998</v>
       </c>
       <c r="E6">
         <v>12</v>
       </c>
       <c r="F6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -577,10 +587,10 @@
         <v>32</v>
       </c>
       <c r="F7">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -597,10 +607,10 @@
         <v>50</v>
       </c>
       <c r="F8">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -620,7 +630,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -637,10 +647,10 @@
         <v>21</v>
       </c>
       <c r="F10">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -660,7 +670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -677,10 +687,10 @@
         <v>53</v>
       </c>
       <c r="F12">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -700,7 +710,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -717,10 +727,10 @@
         <v>75</v>
       </c>
       <c r="F14">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -740,7 +750,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -757,10 +767,10 @@
         <v>3</v>
       </c>
       <c r="F16">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>

</xml_diff>